<commit_message>
chore: Update .gitignore and replace careers.pbix and labs_and_quizzes.xlsx files
</commit_message>
<xml_diff>
--- a/data/Cloud Training/Labs & Quizes/labs_and_quizzes.xlsx
+++ b/data/Cloud Training/Labs & Quizes/labs_and_quizzes.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_4FE271004603599242870A3343FDE641CA53328B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amalitech-my.sharepoint.com/personal/henry_antwi_amalitech_com/Documents/Documents/Power BI Projects/PowerBI_Lab_V2/data/Cloud Training/Labs &amp; Quizes/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_4FE271004603599242870A3343FDE641CA53328B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C362820-9269-485D-AB45-73D1BD3B9E49}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Labs" sheetId="1" r:id="rId1"/>
     <sheet name="Quizzes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -180,7 +185,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,9 +547,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,7 +587,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -614,7 +622,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -649,7 +657,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -684,7 +692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -719,7 +727,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -754,7 +762,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -789,7 +797,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -824,7 +832,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -859,7 +867,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -894,7 +902,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -929,7 +937,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -964,7 +972,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -999,7 +1007,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1034,7 +1042,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1069,7 +1077,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1104,7 +1112,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1139,7 +1147,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1174,7 +1182,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1209,7 +1217,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1244,7 +1252,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1279,7 +1287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1314,7 +1322,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1349,7 +1357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -1384,7 +1392,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -1419,7 +1427,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -1454,7 +1462,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -1489,7 +1497,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1524,7 +1532,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -1559,7 +1567,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -1594,7 +1602,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -1629,7 +1637,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1664,7 +1672,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1699,7 +1707,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -1734,7 +1742,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -1769,7 +1777,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -1804,7 +1812,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>46</v>
       </c>
@@ -1839,7 +1847,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -1874,7 +1882,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -1909,7 +1917,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -1944,7 +1952,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>
@@ -1987,9 +1995,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2024,7 +2032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2059,7 +2067,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2094,7 +2102,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -2129,7 +2137,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -2164,7 +2172,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -2199,7 +2207,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2234,7 +2242,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -2269,7 +2277,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -2304,7 +2312,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2339,7 +2347,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -2374,7 +2382,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -2409,7 +2417,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -2444,7 +2452,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -2479,7 +2487,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -2514,7 +2522,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -2549,7 +2557,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -2584,7 +2592,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -2619,7 +2627,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -2654,7 +2662,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -2689,7 +2697,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -2724,7 +2732,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -2759,7 +2767,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -2794,7 +2802,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -2829,7 +2837,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -2864,7 +2872,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -2899,7 +2907,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -2934,7 +2942,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -2969,7 +2977,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -3004,7 +3012,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -3039,7 +3047,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -3074,7 +3082,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -3109,7 +3117,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -3144,7 +3152,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -3179,7 +3187,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -3214,7 +3222,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -3249,7 +3257,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>46</v>
       </c>
@@ -3284,7 +3292,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -3319,7 +3327,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -3354,7 +3362,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -3389,7 +3397,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>

</xml_diff>